<commit_message>
update Testcase and related content
</commit_message>
<xml_diff>
--- a/test/sprint3/TestDesign Sprint 3.xlsx
+++ b/test/sprint3/TestDesign Sprint 3.xlsx
@@ -1,18 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6354E4BA-3B6F-45DD-9C9D-ED44463E8828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Test Case PBL item 1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Test Case PBL item 16" sheetId="2" r:id="rId6"/>
+    <sheet name="Test Case PBL item 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Case PBL item 16" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="60">
   <si>
     <t>UAT</t>
   </si>
@@ -73,19 +82,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้ UserID แล้วกด "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -108,19 +117,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้เวลาเริ่มต้น แล้วกด "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -140,19 +149,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้เวลาสิ้นสุด แล้วกด "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -175,19 +184,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้เวลาเริ่มต้นและสิ้นสุด แล้วกด "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -207,19 +216,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้ UserID เวลาเริ่มต้นและสิ้นสุด แล้วกด "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -240,19 +249,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้ UserID เวลาเริ่มต้นและสิ้นสุด แล้วกดใช้ "ล้างตัวกรอง" เพื่อล้างข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -273,19 +282,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน Log โดยใช้ UserID ที่ไม่มีในระบบ เวลาเริ่มต้นและสิ้นสุด แล้วกดใช้ "ใช้ตัวกรอง" เพื่อกรองข้อมูล
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -306,19 +315,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">Admin ค้นหาข้อมูลใน ExportLog โดยใช้ เวลาเริ่มต้นและสิ้นสุด จากนั้นกด "ดู" เพื่อดูรายละเอียดการ Export
 </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.เปิดหน้าเว็บไซต์
@@ -340,27 +349,27 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <color rgb="FF000000"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FF000000"/>
-        <sz val="10.0"/>
       </rPr>
       <t>การลบข้อมูลสำเร็จ กรณีไม่เลือกรับข้อมูล</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <color rgb="FF000000"/>
-        <sz val="10.0"/>
       </rPr>
       <t xml:space="preserve">
 1.ล็อคอิน
@@ -381,24 +390,27 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
       </rPr>
       <t>การลบข้อมูลไม่สำเร็จ กรณีกรอกรหัสผ่านผิด</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 1.ล็อคอิน
@@ -418,24 +430,27 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
       </rPr>
       <t>การลบข้อมูล กรณีเลือกรับข้อมูลบางส่วนไปที่อีเมล</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 1.ล็อคอิน
@@ -460,24 +475,27 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
       </rPr>
       <t>การลบข้อมูล กรณีเลือกรับข้อมูลทั้งหมดไปที่อีเมล</t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
 1.ล็อคอิน
@@ -488,73 +506,124 @@
 6.กดปุ่ม “ยืนยันการลบ”</t>
     </r>
   </si>
+  <si>
+    <t>TC01-09</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Admin ค้นหาข้อมูลใน Traffic-Log จากนั้นกด "Export" เพื่อทำการส่งออกข้อมูลไปเก็บไว้ในเครื่อง
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">
+1.เปิดหน้าเว็บไซต์
+2.ไปยังหน้าเข้าสู่ระบบ
+3.เข้าสู่ระบบโดยใช้ Admin ID
+4.ไปยังหน้า Traffic-Log
+5. กดปุ่ม "Export" เพื่อทำการส่งออกข้อมูล</t>
+    </r>
+  </si>
+  <si>
+    <t>ได้รับไฟล์ Traffic-Log ไปเก็บไว้ใน โฟล์เดอร์ที่กำหนดไว้</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="165" formatCode="d mmmm yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d\ mmmm\ yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18.0"/>
-      <color theme="1"/>
-      <name val="Sarabun"/>
-    </font>
-    <font/>
-    <font>
-      <sz val="18.0"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Sarabun"/>
     </font>
     <font>
-      <sz val="16.0"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Sarabun"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Sarabun"/>
     </font>
     <font>
       <u/>
-      <sz val="18.0"/>
+      <sz val="18"/>
       <color rgb="FF0000FF"/>
       <name val="Sarabun"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="16.0"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="&quot;TH SarabunPSK&quot;"/>
     </font>
     <font>
-      <sz val="18.0"/>
+      <sz val="18"/>
       <color rgb="FFFF0000"/>
       <name val="Sarabun"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -564,7 +633,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -609,28 +678,40 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
-    <border/>
+  <borders count="10">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -640,6 +721,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -654,6 +736,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -665,6 +748,8 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -673,6 +758,9 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -681,145 +769,159 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="39">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="5" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="5" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1009,289 +1111,305 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H998"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="25.5"/>
-    <col customWidth="1" min="2" max="2" width="21.5"/>
-    <col customWidth="1" min="3" max="3" width="27.38"/>
-    <col customWidth="1" min="4" max="4" width="26.13"/>
-    <col customWidth="1" min="5" max="5" width="23.88"/>
-    <col customWidth="1" min="6" max="6" width="39.25"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="26.109375" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="39.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="33" customHeight="1">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="24"/>
     </row>
-    <row r="2" ht="15.0" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+    <row r="2" spans="1:6" ht="15" customHeight="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
-    <row r="3" ht="24.0" customHeight="1">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:6" ht="24" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="26"/>
+      <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="3"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="24"/>
     </row>
-    <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:6" ht="24" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="9">
-        <v>244425.0</v>
-      </c>
-      <c r="F4" s="3"/>
+      <c r="E4" s="33">
+        <v>244425</v>
+      </c>
+      <c r="F4" s="24"/>
     </row>
-    <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="5" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="24"/>
     </row>
-    <row r="6" ht="24.0" customHeight="1">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:6" ht="24" customHeight="1">
+      <c r="A6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="24"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
     </row>
-    <row r="8" ht="39.0" customHeight="1">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:6" ht="39" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="191.25" customHeight="1">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:6" ht="191.25" customHeight="1">
+      <c r="A9" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="195.0" customHeight="1">
-      <c r="A10" s="19"/>
-      <c r="B10" s="15" t="s">
+    <row r="10" spans="1:6" ht="195" customHeight="1">
+      <c r="A10" s="38"/>
+      <c r="B10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="208.5" customHeight="1">
-      <c r="A11" s="19"/>
-      <c r="B11" s="15" t="s">
+    <row r="11" spans="1:6" ht="208.5" customHeight="1">
+      <c r="A11" s="38"/>
+      <c r="B11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" ht="213.0" customHeight="1">
-      <c r="A12" s="19"/>
-      <c r="B12" s="15" t="s">
+    <row r="12" spans="1:6" ht="213" customHeight="1">
+      <c r="A12" s="38"/>
+      <c r="B12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" ht="246.0" customHeight="1">
-      <c r="A13" s="19"/>
-      <c r="B13" s="15" t="s">
+    <row r="13" spans="1:6" ht="246" customHeight="1">
+      <c r="A13" s="38"/>
+      <c r="B13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" ht="225.0" customHeight="1">
-      <c r="A14" s="19"/>
-      <c r="B14" s="15" t="s">
+    <row r="14" spans="1:6" ht="225" customHeight="1">
+      <c r="A14" s="38"/>
+      <c r="B14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" ht="261.0" customHeight="1">
-      <c r="A15" s="19"/>
-      <c r="B15" s="15" t="s">
+    <row r="15" spans="1:6" ht="261" customHeight="1">
+      <c r="A15" s="38"/>
+      <c r="B15" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" ht="207.75" customHeight="1">
-      <c r="A16" s="20"/>
-      <c r="B16" s="15" t="s">
+    <row r="16" spans="1:6" ht="207.75" customHeight="1">
+      <c r="A16" s="38"/>
+      <c r="B16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" ht="234.0" customHeight="1">
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
+    <row r="17" spans="1:8" ht="234" customHeight="1">
+      <c r="A17" s="38"/>
+      <c r="B17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
     </row>
-    <row r="18" ht="230.25" customHeight="1"/>
-    <row r="19" ht="165.75" customHeight="1"/>
-    <row r="20" ht="198.0" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="18" spans="1:8" ht="230.25" customHeight="1"/>
+    <row r="19" spans="1:8" ht="165.75" customHeight="1"/>
+    <row r="20" spans="1:8" ht="198" customHeight="1"/>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2260,9 +2378,9 @@
     <row r="998" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A9:A17"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:F6"/>
-    <mergeCell ref="A9:A16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
@@ -2271,233 +2389,230 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="E5:F5"/>
   </mergeCells>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:F16">
+  <phoneticPr fontId="14" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:F17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C6"/>
+    <hyperlink ref="C6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H998"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="25.5"/>
-    <col customWidth="1" min="2" max="2" width="21.5"/>
-    <col customWidth="1" min="3" max="3" width="27.38"/>
-    <col customWidth="1" min="4" max="4" width="26.13"/>
-    <col customWidth="1" min="5" max="5" width="23.88"/>
-    <col customWidth="1" min="6" max="6" width="39.25"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="26.109375" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="39.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="33" customHeight="1">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="24"/>
     </row>
-    <row r="2" ht="15.0" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+    <row r="2" spans="1:6" ht="15" customHeight="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
-    <row r="3" ht="24.0" customHeight="1">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:6" ht="24" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="26"/>
+      <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="3"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="24"/>
     </row>
-    <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:6" ht="24" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="23">
-        <v>244425.0</v>
-      </c>
-      <c r="F4" s="3"/>
+      <c r="E4" s="36">
+        <v>244425</v>
+      </c>
+      <c r="F4" s="24"/>
     </row>
-    <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="24" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="26"/>
+      <c r="F5" s="10"/>
     </row>
-    <row r="6" ht="24.0" customHeight="1">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:6" ht="24" customHeight="1">
+      <c r="A6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="24"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
     </row>
-    <row r="8" ht="39.0" customHeight="1">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:6" ht="39" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="191.25" customHeight="1">
-      <c r="A9" s="27" t="s">
+    <row r="9" spans="1:6" ht="191.25" customHeight="1">
+      <c r="A9" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="31" t="s">
+      <c r="E9" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="195.0" customHeight="1">
-      <c r="A10" s="19"/>
-      <c r="B10" s="32" t="s">
+    <row r="10" spans="1:6" ht="195" customHeight="1">
+      <c r="A10" s="27"/>
+      <c r="B10" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F10" s="35" t="s">
+      <c r="F10" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="208.5" customHeight="1">
-      <c r="A11" s="19"/>
-      <c r="B11" s="36" t="s">
+    <row r="11" spans="1:6" ht="208.5" customHeight="1">
+      <c r="A11" s="27"/>
+      <c r="B11" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" ht="213.0" customHeight="1">
-      <c r="A12" s="20"/>
-      <c r="B12" s="38" t="s">
+    <row r="12" spans="1:6" ht="213" customHeight="1">
+      <c r="A12" s="28"/>
+      <c r="B12" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F12" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" ht="246.0" customHeight="1"/>
-    <row r="14" ht="225.0" customHeight="1"/>
-    <row r="15" ht="261.0" customHeight="1"/>
-    <row r="16" ht="207.75" customHeight="1"/>
-    <row r="17" ht="234.0" customHeight="1">
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
+    <row r="13" spans="1:6" ht="246" customHeight="1"/>
+    <row r="14" spans="1:6" ht="225" customHeight="1"/>
+    <row r="15" spans="1:6" ht="261" customHeight="1"/>
+    <row r="16" spans="1:6" ht="207.75" customHeight="1"/>
+    <row r="17" spans="7:8" ht="234" customHeight="1">
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
     </row>
-    <row r="18" ht="230.25" customHeight="1"/>
-    <row r="19" ht="165.75" customHeight="1"/>
-    <row r="20" ht="198.0" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="18" spans="7:8" ht="230.25" customHeight="1"/>
+    <row r="19" spans="7:8" ht="165.75" customHeight="1"/>
+    <row r="20" spans="7:8" ht="198" customHeight="1"/>
+    <row r="21" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="22" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="23" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="24" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="25" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="26" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="27" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="28" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="29" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="30" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="31" spans="7:8" ht="15.75" customHeight="1"/>
+    <row r="32" spans="7:8" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -3476,17 +3591,15 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
   </mergeCells>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:F12">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F9:F12" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C6"/>
+    <hyperlink ref="C6" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>